<commit_message>
feat: new peer asssesment
</commit_message>
<xml_diff>
--- a/My_Professional_Reviews/UAS-5_Skor.xlsx
+++ b/My_Professional_Reviews/UAS-5_Skor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\all-about-me\My_Professional_Reviews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF624EE-6643-4DE0-8790-527A83ADDF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8DAA21-09BD-4EEE-B001-C933DE64C426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
   </bookViews>
   <sheets>
     <sheet name="UAS_1_My_Concepts" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -121,14 +121,30 @@
   <si>
     <t>M. Abizzar Gamadrian</t>
   </si>
+  <si>
+    <t>Tyara Penelope Lumban Gaol</t>
+  </si>
+  <si>
+    <t>Mahesa Fadhillah Andre</t>
+  </si>
+  <si>
+    <t>Muhammad Raihaan Perdana</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -190,14 +206,16 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -643,6 +661,12 @@
       <c r="AP3" s="4"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>18224122</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -656,9 +680,27 @@
       <c r="AP4" s="4"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G5" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A5" s="2">
+        <v>13523140</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
@@ -669,9 +711,27 @@
       <c r="AP5" s="4"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G6" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A6" s="2">
+        <v>13523124</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L6" s="4"/>
       <c r="Q6" s="4"/>
@@ -1677,6 +1737,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1811,6 +1872,12 @@
       <c r="AP3" s="4"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>18224122</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1824,9 +1891,27 @@
       <c r="AP4" s="4"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G5" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A5" s="7">
+        <v>13523140</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
@@ -1837,9 +1922,27 @@
       <c r="AP5" s="4"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G6" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A6" s="2">
+        <v>13523124</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L6" s="4"/>
       <c r="Q6" s="4"/>
@@ -2979,6 +3082,12 @@
       <c r="AP3" s="4"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>18224122</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2992,9 +3101,27 @@
       <c r="AP4" s="4"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G5" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A5" s="7">
+        <v>13523140</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>4.9000000000000004</v>
       </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
@@ -3005,9 +3132,27 @@
       <c r="AP5" s="4"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G6" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A6" s="2">
+        <v>13523124</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L6" s="4"/>
       <c r="Q6" s="4"/>
@@ -4147,6 +4292,12 @@
       <c r="AP3" s="4"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>18224122</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4160,9 +4311,27 @@
       <c r="AP4" s="4"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G5" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A5" s="7">
+        <v>13523140</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L5" s="4"/>
       <c r="Q5" s="4"/>
@@ -4173,9 +4342,27 @@
       <c r="AP5" s="4"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="G6" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="A6" s="2">
+        <v>13523124</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F6" s="2">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>4.9000000000000004</v>
       </c>
       <c r="L6" s="4"/>
       <c r="Q6" s="4"/>

</xml_diff>

<commit_message>
feat: final peer assesment
</commit_message>
<xml_diff>
--- a/My_Professional_Reviews/UAS-5_Skor.xlsx
+++ b/My_Professional_Reviews/UAS-5_Skor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\all-about-me\My_Professional_Reviews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8DAA21-09BD-4EEE-B001-C933DE64C426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2BD707-0522-4385-9FC5-4E4BB34A14AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
   </bookViews>
   <sheets>
     <sheet name="UAS_1_My_Concepts" sheetId="2" r:id="rId1"/>
@@ -667,9 +667,21 @@
       <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C4" s="2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>5</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L4" s="4"/>
       <c r="Q4" s="4"/>
@@ -1878,9 +1890,21 @@
       <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C4" s="2">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>4</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
       </c>
       <c r="L4" s="4"/>
       <c r="Q4" s="4"/>
@@ -3088,9 +3112,21 @@
       <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C4" s="2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>5</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L4" s="4"/>
       <c r="Q4" s="4"/>
@@ -4298,9 +4334,21 @@
       <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="C4" s="2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>5</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="L4" s="4"/>
       <c r="Q4" s="4"/>

</xml_diff>